<commit_message>
Added loop for calculating strain
</commit_message>
<xml_diff>
--- a/Code/Matlab/Analysis/Dynamic_Simulation/Max Strain Computation.xlsx
+++ b/Code/Matlab/Analysis/Dynamic_Simulation/Max Strain Computation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mnstr\Documents\GitHub\Quad\Code\Matlab\Analysis\Dynamic_Simulation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7929F1CF-AA64-4B9E-A034-339B2515FFC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8019E88F-1F0D-4E3D-A0A4-87777004C4AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{B58E221A-B97F-48A6-8396-F4ED8454BDD2}"/>
+    <workbookView xWindow="36075" yWindow="0" windowWidth="12825" windowHeight="12165" xr2:uid="{B58E221A-B97F-48A6-8396-F4ED8454BDD2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -490,7 +490,7 @@
     <col min="11" max="11" width="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -525,12 +525,12 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
       <c r="B2">
-        <f>K2/F2</f>
+        <f>ABS(K2/F2)</f>
         <v>5.5922892200401322E-3</v>
       </c>
       <c r="C2">
@@ -564,12 +564,12 @@
         <v>1.6999999999999999E-3</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
       <c r="B3">
-        <f t="shared" ref="B3:B10" si="0">K3/F3</f>
+        <f t="shared" ref="B3:B10" si="0">ABS(K3/F3)</f>
         <v>3.3333333333148145E-4</v>
       </c>
       <c r="C3">
@@ -603,24 +603,24 @@
         <v>1E-4</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
       <c r="B4">
-        <f t="shared" si="0"/>
-        <v>6.4694487710838288E-3</v>
+        <f>ABS(K4/F4)+L4</f>
+        <v>5.8969448771083829E-2</v>
       </c>
       <c r="C4">
         <v>0</v>
       </c>
       <c r="D4" s="2">
         <f t="shared" si="1"/>
-        <v>192.34752700822574</v>
+        <v>317.28272365760148</v>
       </c>
       <c r="E4" s="3">
         <f t="shared" si="2"/>
-        <v>27.896668166530205</v>
+        <v>46.016348608789194</v>
       </c>
       <c r="F4">
         <v>0.24731627942575879</v>
@@ -641,25 +641,28 @@
       <c r="K4">
         <v>1.6000000000000001E-3</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L4">
+        <v>5.2499999999999998E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
       <c r="B5">
-        <f t="shared" si="0"/>
-        <v>7.2784618184023779E-3</v>
+        <f t="shared" ref="B5:B7" si="4">ABS(K5/F5)+L5</f>
+        <v>5.9778461818402379E-2</v>
       </c>
       <c r="C5">
         <v>1.3039000000000001</v>
       </c>
       <c r="D5" s="2">
         <f t="shared" si="1"/>
-        <v>196.4235612918217</v>
+        <v>321.55935909668841</v>
       </c>
       <c r="E5" s="3">
         <f t="shared" si="2"/>
-        <v>28.487826148197492</v>
+        <v>46.63660030408824</v>
       </c>
       <c r="F5">
         <v>0.247305</v>
@@ -680,25 +683,28 @@
       <c r="K5">
         <v>1.8E-3</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L5">
+        <v>5.2499999999999998E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
       <c r="B6">
-        <f t="shared" si="0"/>
-        <v>1.1688729142923936E-3</v>
+        <f t="shared" si="4"/>
+        <v>3.7468872914292392E-2</v>
       </c>
       <c r="C6">
         <v>2.1206999999999998</v>
       </c>
       <c r="D6" s="2">
         <f t="shared" si="1"/>
-        <v>180.46924292004275</v>
+        <v>270.10889892929441</v>
       </c>
       <c r="E6" s="3">
         <f t="shared" si="2"/>
-        <v>26.173929357511639</v>
+        <v>39.174604630789617</v>
       </c>
       <c r="F6">
         <v>0.17110500000000001</v>
@@ -719,25 +725,28 @@
       <c r="K6">
         <v>2.0000000000000001E-4</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L6">
+        <v>3.6299999999999999E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>10</v>
       </c>
       <c r="B7">
-        <f t="shared" si="0"/>
-        <v>2.571520411443266E-2</v>
+        <f t="shared" si="4"/>
+        <v>6.2015204114432662E-2</v>
       </c>
       <c r="C7">
         <v>0</v>
       </c>
       <c r="D7" s="2">
         <f t="shared" si="1"/>
-        <v>240.00563230808422</v>
+        <v>324.74843180104801</v>
       </c>
       <c r="E7" s="3">
         <f t="shared" si="2"/>
-        <v>34.808648630614101</v>
+        <v>47.099119913132419</v>
       </c>
       <c r="F7">
         <v>0.17110500000000001</v>
@@ -758,8 +767,11 @@
       <c r="K7">
         <v>4.4000000000000003E-3</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L7">
+        <v>3.6299999999999999E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -798,7 +810,7 @@
         <v>3.3099999999999997E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -837,7 +849,7 @@
         <v>2.3E-3</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -876,7 +888,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>18</v>
       </c>
@@ -888,7 +900,7 @@
         <v>3.3099999999999796E-3</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>19</v>
       </c>
@@ -1009,27 +1021,24 @@
       <c r="K24">
         <v>3.2000000000000002E-3</v>
       </c>
-      <c r="L24">
-        <v>8.5000000000000006E-2</v>
-      </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>6</v>
       </c>
       <c r="B25">
-        <f t="shared" ref="B25:B32" si="4">ABS(K25/F25)</f>
+        <f t="shared" ref="B25:B32" si="5">ABS(K25/F25)</f>
         <v>1.9999999999888888E-2</v>
       </c>
       <c r="C25">
         <v>10.006</v>
       </c>
       <c r="D25" s="2">
-        <f t="shared" ref="D25:D32" si="5">($B$15+$B$16*TAN($B$17*(B25/($B$19*J25+0.17))+$B$18)+($B$20*J25)+($B$21*1))/1000</f>
+        <f t="shared" ref="D25:D32" si="6">($B$15+$B$16*TAN($B$17*(B25/($B$19*J25+0.17))+$B$18)+($B$20*J25)+($B$21*1))/1000</f>
         <v>503.99397398166855</v>
       </c>
       <c r="E25" s="3">
-        <f t="shared" ref="E25:E32" si="6">D25/6.895</f>
+        <f t="shared" ref="E25:E32" si="7">D25/6.895</f>
         <v>73.09557273120646</v>
       </c>
       <c r="F25">
@@ -1042,7 +1051,7 @@
         <v>0.38486821453293901</v>
       </c>
       <c r="I25">
-        <f t="shared" ref="I25:I32" si="7">G25-H25</f>
+        <f t="shared" ref="I25:I32" si="8">G25-H25</f>
         <v>4.8578660357370129E-3</v>
       </c>
       <c r="J25">
@@ -1057,19 +1066,19 @@
         <v>7</v>
       </c>
       <c r="B26">
-        <f t="shared" si="4"/>
-        <v>4.0434054819273929E-3</v>
+        <f>ABS(K26/F26)+L26</f>
+        <v>5.6543405481927392E-2</v>
       </c>
       <c r="C26">
         <v>0</v>
       </c>
       <c r="D26" s="2">
-        <f t="shared" si="5"/>
-        <v>185.97939553309129</v>
+        <f t="shared" si="6"/>
+        <v>311.63328594199021</v>
       </c>
       <c r="E26" s="3">
-        <f t="shared" si="6"/>
-        <v>26.973081295589747</v>
+        <f t="shared" si="7"/>
+        <v>45.196995785640354</v>
       </c>
       <c r="F26">
         <v>0.24731627942575879</v>
@@ -1081,7 +1090,7 @@
         <v>0.329635163815787</v>
       </c>
       <c r="I26">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1.217037473645699E-2</v>
       </c>
       <c r="J26">
@@ -1091,7 +1100,7 @@
         <v>-1E-3</v>
       </c>
       <c r="L26">
-        <v>8.5000000000000006E-2</v>
+        <v>5.2499999999999998E-2</v>
       </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.25">
@@ -1099,19 +1108,19 @@
         <v>8</v>
       </c>
       <c r="B27">
-        <f t="shared" si="4"/>
-        <v>5.6610258587574047E-3</v>
+        <f>ABS(K27/F27)+L27</f>
+        <v>5.8161025858757404E-2</v>
       </c>
       <c r="C27">
         <v>1.3039000000000001</v>
       </c>
       <c r="D27" s="2">
-        <f t="shared" si="5"/>
-        <v>620.70347512140404</v>
+        <f t="shared" si="6"/>
+        <v>2527.9490085222319</v>
       </c>
       <c r="E27" s="3">
-        <f t="shared" si="6"/>
-        <v>90.022258900856286</v>
+        <f t="shared" si="7"/>
+        <v>366.63509913302858</v>
       </c>
       <c r="F27">
         <v>0.247305</v>
@@ -1123,7 +1132,7 @@
         <v>0.32037392471992399</v>
       </c>
       <c r="I27">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1.3064431618028005E-2</v>
       </c>
       <c r="J27">
@@ -1131,6 +1140,9 @@
       </c>
       <c r="K27">
         <v>1.4E-3</v>
+      </c>
+      <c r="L27">
+        <v>5.2499999999999998E-2</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
@@ -1138,19 +1150,19 @@
         <v>9</v>
       </c>
       <c r="B28">
-        <f t="shared" si="4"/>
-        <v>2.162414891440928E-2</v>
+        <f>ABS(K28/F28)+L28</f>
+        <v>5.7924148914409279E-2</v>
       </c>
       <c r="C28">
         <v>2.1206999999999998</v>
       </c>
       <c r="D28" s="2">
-        <f t="shared" si="5"/>
-        <v>447.72720039872939</v>
+        <f t="shared" si="6"/>
+        <v>579.13228181781972</v>
       </c>
       <c r="E28" s="3">
-        <f t="shared" si="6"/>
-        <v>64.935054445065902</v>
+        <f t="shared" si="7"/>
+        <v>83.993079306427816</v>
       </c>
       <c r="F28">
         <v>0.17110500000000001</v>
@@ -1162,7 +1174,7 @@
         <v>0.20866553670100499</v>
       </c>
       <c r="I28">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>5.1257493845530133E-3</v>
       </c>
       <c r="J28">
@@ -1172,7 +1184,7 @@
         <v>3.7000000000000002E-3</v>
       </c>
       <c r="L28">
-        <v>8.5000000000000006E-2</v>
+        <v>3.6299999999999999E-2</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
@@ -1180,19 +1192,19 @@
         <v>10</v>
       </c>
       <c r="B29">
-        <f t="shared" si="4"/>
-        <v>0</v>
+        <f>ABS(K29/F29)+L29</f>
+        <v>3.6299999999999999E-2</v>
       </c>
       <c r="C29">
         <v>0</v>
       </c>
       <c r="D29" s="2">
-        <f t="shared" si="5"/>
-        <v>174.5345875730934</v>
+        <f t="shared" si="6"/>
+        <v>264.46828339605253</v>
       </c>
       <c r="E29" s="3">
-        <f t="shared" si="6"/>
-        <v>25.313210670499409</v>
+        <f t="shared" si="7"/>
+        <v>38.356531311972816</v>
       </c>
       <c r="F29">
         <v>0.17110500000000001</v>
@@ -1204,7 +1216,7 @@
         <v>0.21235836428733601</v>
       </c>
       <c r="I29">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>5.7817633340679908E-3</v>
       </c>
       <c r="J29">
@@ -1212,6 +1224,9 @@
       </c>
       <c r="K29">
         <v>0</v>
+      </c>
+      <c r="L29">
+        <v>3.6299999999999999E-2</v>
       </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.25">
@@ -1219,18 +1234,18 @@
         <v>11</v>
       </c>
       <c r="B30">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>8.5688334390156135E-2</v>
       </c>
       <c r="C30">
         <v>7.0512000000000005E-2</v>
       </c>
       <c r="D30" s="2">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>808.07102455253971</v>
       </c>
       <c r="E30" s="3">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>117.1966678103756</v>
       </c>
       <c r="F30">
@@ -1243,7 +1258,7 @@
         <v>0.30457987255206198</v>
       </c>
       <c r="I30">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>3.5854826738452028E-2</v>
       </c>
       <c r="J30">
@@ -1258,18 +1273,18 @@
         <v>12</v>
       </c>
       <c r="B31">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>7.6091240938458649E-2</v>
       </c>
       <c r="C31">
         <v>0.35621999999999998</v>
       </c>
       <c r="D31" s="2">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>777.90502951295389</v>
       </c>
       <c r="E31" s="3">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>112.82161414256039</v>
       </c>
       <c r="F31">
@@ -1282,7 +1297,7 @@
         <v>0.30389949865746102</v>
       </c>
       <c r="I31">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1.5510458449289999E-2</v>
       </c>
       <c r="J31">
@@ -1297,18 +1312,18 @@
         <v>13</v>
       </c>
       <c r="B32">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>3.0746659957427171E-2</v>
       </c>
       <c r="C32">
         <v>0.90895000000000004</v>
       </c>
       <c r="D32" s="2">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>545.4943998325034</v>
       </c>
       <c r="E32" s="3">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>79.11448873567852</v>
       </c>
       <c r="F32">
@@ -1321,7 +1336,7 @@
         <v>0.305372064749449</v>
       </c>
       <c r="I32">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1.7702751174533016E-2</v>
       </c>
       <c r="J32">

</xml_diff>